<commit_message>
Single sentence all runs.
</commit_message>
<xml_diff>
--- a/results/single_sentence_comparison.xlsx
+++ b/results/single_sentence_comparison.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mdodovic\Desktop\LLM-HS-Detector\HateSpeech-LLM-Detector\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762B7C79-B360-49BA-8487-9AF7AD4EF075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B05ADEDD-F311-4F5F-92B3-A5F847BCD203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4410" yWindow="2385" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="300" yWindow="3225" windowWidth="21600" windowHeight="12645" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="One Prompt" sheetId="1" r:id="rId1"/>
-    <sheet name="Two Prompts" sheetId="2" r:id="rId2"/>
+    <sheet name="Two Prompts" sheetId="3" r:id="rId1"/>
+    <sheet name="One Prompt" sheetId="4" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="24">
   <si>
     <t>model</t>
   </si>
@@ -89,22 +89,23 @@
   </si>
   <si>
     <t>qwen3</t>
+  </si>
+  <si>
+    <t>mistral</t>
+  </si>
+  <si>
+    <t>deepseek-r1</t>
+  </si>
+  <si>
+    <t>phi3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -125,7 +126,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -148,31 +149,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -476,8 +459,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:S6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -544,37 +527,37 @@
         <v>19</v>
       </c>
       <c r="B2">
-        <v>0.77777777777777779</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="F2">
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="G2">
-        <v>0.375</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H2">
-        <v>0.3</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="I2">
-        <v>0.25</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="J2">
-        <v>0.66666666666666663</v>
+        <v>0.5</v>
       </c>
       <c r="K2">
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="L2">
-        <v>0.33333333333333331</v>
+        <v>0.5</v>
       </c>
       <c r="M2">
         <v>0.5</v>
@@ -600,40 +583,40 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3">
-        <v>0.88888888888888884</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D3">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>0.8571428571428571</v>
+        <v>0.8</v>
       </c>
       <c r="F3">
-        <v>0.77777777777777779</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="G3">
-        <v>0.45833333333333343</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="H3">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="I3">
-        <v>0.47727272727272729</v>
+        <v>0.26666666666666672</v>
       </c>
       <c r="J3">
-        <v>0.68518518518518523</v>
+        <v>0.44444444444444442</v>
       </c>
       <c r="K3">
-        <v>0.77777777777777779</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="L3">
-        <v>0.72727272727272718</v>
+        <v>0.35555555555555562</v>
       </c>
       <c r="M3">
         <v>0.5</v>
@@ -657,72 +640,249 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="C4">
+        <v>0.8</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="F4">
+        <v>0.2</v>
+      </c>
+      <c r="G4">
+        <v>0.2</v>
+      </c>
+      <c r="H4">
+        <v>0.1</v>
+      </c>
+      <c r="I4">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="J4">
+        <v>0.4</v>
+      </c>
+      <c r="K4">
+        <v>0.2</v>
+      </c>
+      <c r="L4">
+        <v>0.26666666666666672</v>
+      </c>
+      <c r="M4">
+        <v>0.5</v>
+      </c>
+      <c r="N4">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="O4">
+        <v>0.16666666666666671</v>
+      </c>
+      <c r="P4">
+        <v>0.22222222222222221</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>0.5</v>
+      </c>
+      <c r="S4">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0.25</v>
+      </c>
+      <c r="E5">
+        <v>0.4</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>0.5</v>
+      </c>
+      <c r="G6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="H6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="I6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="J6">
+        <v>0.5</v>
+      </c>
+      <c r="K6">
+        <v>0.5</v>
+      </c>
+      <c r="L6">
+        <v>0.5</v>
+      </c>
+      <c r="M6">
+        <v>0.5</v>
+      </c>
+      <c r="N6">
+        <v>0.5</v>
+      </c>
+      <c r="O6">
+        <v>0.25</v>
+      </c>
+      <c r="P6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>0.5</v>
+      </c>
+      <c r="S6">
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:S3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:S6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
@@ -731,37 +891,37 @@
         <v>19</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F2">
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="G2">
-        <v>0.33333333333333331</v>
+        <v>0.375</v>
       </c>
       <c r="H2">
-        <v>0.33333333333333331</v>
+        <v>0.3</v>
       </c>
       <c r="I2">
-        <v>0.33333333333333331</v>
+        <v>0.25</v>
       </c>
       <c r="J2">
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="K2">
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="L2">
-        <v>0.5</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="M2">
         <v>0.5</v>
@@ -787,60 +947,237 @@
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>0.75</v>
+      </c>
+      <c r="E3">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F3">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="G3">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="H3">
+        <v>0.5</v>
+      </c>
+      <c r="I3">
+        <v>0.47863247863247871</v>
+      </c>
+      <c r="J3">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="K3">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="L3">
+        <v>0.57549857549857553</v>
+      </c>
+      <c r="M3">
+        <v>0.75</v>
+      </c>
+      <c r="N3">
+        <v>0.5</v>
+      </c>
+      <c r="O3">
+        <v>0.375</v>
+      </c>
+      <c r="P3">
+        <v>0.42857142857142849</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>0.75</v>
+      </c>
+      <c r="S3">
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="C4">
+        <v>0.8</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="F4">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="G4">
+        <v>0.4</v>
+      </c>
+      <c r="H4">
+        <v>0.4</v>
+      </c>
+      <c r="I4">
+        <v>0.4</v>
+      </c>
+      <c r="J4">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="K4">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="L4">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="M4">
+        <v>0.25</v>
+      </c>
+      <c r="N4">
+        <v>0.25</v>
+      </c>
+      <c r="O4">
+        <v>6.25E-2</v>
+      </c>
+      <c r="P4">
+        <v>0.1</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>0.25</v>
+      </c>
+      <c r="S4">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="E5">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="F5">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="G5">
+        <v>0.41666666666666657</v>
+      </c>
+      <c r="H5">
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="I5">
+        <v>0.34848484848484851</v>
+      </c>
+      <c r="J5">
+        <v>0.59259259259259256</v>
+      </c>
+      <c r="K5">
+        <v>0.55555555555555558</v>
+      </c>
+      <c r="L5">
+        <v>0.55218855218855223</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
-      <c r="F3">
-        <v>0.5</v>
-      </c>
-      <c r="G3">
+      <c r="B6">
+        <v>0.88888888888888884</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>0.75</v>
+      </c>
+      <c r="E6">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="F6">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="G6">
+        <v>0.45833333333333343</v>
+      </c>
+      <c r="H6">
+        <v>0.5</v>
+      </c>
+      <c r="I6">
+        <v>0.47727272727272729</v>
+      </c>
+      <c r="J6">
+        <v>0.68518518518518523</v>
+      </c>
+      <c r="K6">
+        <v>0.77777777777777779</v>
+      </c>
+      <c r="L6">
+        <v>0.72727272727272718</v>
+      </c>
+      <c r="M6">
+        <v>0.5</v>
+      </c>
+      <c r="N6">
+        <v>0.5</v>
+      </c>
+      <c r="O6">
         <v>0.25</v>
       </c>
-      <c r="H3">
-        <v>0.25</v>
-      </c>
-      <c r="I3">
-        <v>0.25</v>
-      </c>
-      <c r="J3">
-        <v>0.5</v>
-      </c>
-      <c r="K3">
-        <v>0.5</v>
-      </c>
-      <c r="L3">
-        <v>0.5</v>
-      </c>
-      <c r="M3">
-        <v>0.5</v>
-      </c>
-      <c r="N3">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="O3">
-        <v>0.16666666666666671</v>
-      </c>
-      <c r="P3">
-        <v>0.22222222222222221</v>
-      </c>
-      <c r="Q3">
-        <v>1</v>
-      </c>
-      <c r="R3">
-        <v>0.5</v>
-      </c>
-      <c r="S3">
+      <c r="P6">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>0.5</v>
+      </c>
+      <c r="S6">
         <v>0.66666666666666663</v>
       </c>
     </row>

</xml_diff>